<commit_message>
Vertrags-Soll 38 h x 18 Wochen in der Wochenuebersicht
Unter der Wochentabelle steht jetzt der Abgleich mit dem Vertrag:
Soll 38,0 h/Woche x 18 Wochen = 684,00 h, Ist 709,50 h, Differenz
+25,50 h. Die Stunden selbst bleiben unveraendert.

Die Spalte "Soll" in der Tabelle bleibt der Wochenvergleich (38,0 h
anteilig je Anwesenheitstag, Hochschul- und Pruefungstage als halber
Tag). Zwei Fussnoten trennen die beiden Groessen und erklaeren, warum
der Schnitt von 32,25 h/Woche niedriger wirkt als der Vertrag: er teilt
ueber alle 22 Kalenderwochen, also einschliesslich der Wochen mit
Feiertag, Krankheit oder vollem Hochschultag. Die Spaltenbeschriftung
heisst deshalb jetzt "Ø je Kalenderwoche".

Geprueft: Nachweis, Monatsblaetter und Wochenuebersicht ergeben
uebereinstimmend 709,50 h; der Vertragsblock rechnet 684,00 / 709,50 /
+25,50; 0 Abweichungen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U4BNk3uadsQpTDXBqWzPi1
</commit_message>
<xml_diff>
--- a/hochschule/Hassine_3399727_Zeiterfassung.xlsx
+++ b/hochschule/Hassine_3399727_Zeiterfassung.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Juli" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Wochenübersicht'!$A$1:$G$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Wochenübersicht'!$A$1:$G$36</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'März'!$A$1:$G$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'April'!$A$1:$G$43</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'Mai'!$A$1:$G$43</definedName>
@@ -34,7 +34,7 @@
     <numFmt numFmtId="166" formatCode="HH:MM"/>
     <numFmt numFmtId="167" formatCode="+0.00;-0.00;0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -106,6 +106,11 @@
       <i val="1"/>
       <color rgb="00595959"/>
       <sz val="8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="6">
@@ -181,7 +186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -218,7 +223,19 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="2" fontId="13" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -619,7 +636,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1351,21 +1368,65 @@
     <row r="28">
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>Ø je Woche</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>Wochen über einen Monatswechsel sind hier vollständig zusammengefasst; in den Monatsblättern erscheinen sie anteilig.</t>
+          <t>Ø je Kalenderwoche</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="14" t="inlineStr">
         <is>
-          <t>Soll = 38,0 h/Woche, anteilig je Anwesenheitstag. Vorlesungs-, Praktikums- und Prüfungstage zählen als halber Tag, weil der Vormittag an der OTH war.</t>
+          <t>Soll laut Vertrag</t>
+        </is>
+      </c>
+      <c r="D30" s="15" t="n">
+        <v>684</v>
+      </c>
+      <c r="E30" s="16" t="inlineStr">
+        <is>
+          <t>38,0 h/Woche × 18 Wochen</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="14" t="inlineStr">
+        <is>
+          <t>Ist laut Tätigkeitsnachweis</t>
+        </is>
+      </c>
+      <c r="D31" s="15">
+        <f>D27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>Differenz</t>
+        </is>
+      </c>
+      <c r="D32" s="18">
+        <f>D27-684.0</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>Wochen über einen Monatswechsel sind hier vollständig zusammengefasst; in den Monatsblättern erscheinen sie anteilig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>Spalte Soll = 38,0 h/Woche, anteilig je Anwesenheitstag. Vorlesungs-, Praktikums- und Prüfungstage zählen als halber Tag, weil der Vormittag an der OTH war.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>Ø je Kalenderwoche rechnet über alle 22 Wochen des Zeitraums, also einschließlich der Wochen mit Feiertag, Krankheit oder Hochschultag.</t>
         </is>
       </c>
     </row>
@@ -1459,19 +1520,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr">
+      <c r="A5" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B5" s="16" t="n">
+      <c r="B5" s="20" t="n">
         <v>46082</v>
       </c>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="15" t="n"/>
-      <c r="E5" s="15" t="n"/>
-      <c r="F5" s="15" t="n"/>
-      <c r="G5" s="17" t="inlineStr">
+      <c r="C5" s="19" t="n"/>
+      <c r="D5" s="19" t="n"/>
+      <c r="E5" s="19" t="n"/>
+      <c r="F5" s="19" t="n"/>
+      <c r="G5" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
@@ -1483,16 +1544,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="22" t="n">
         <v>46083</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="23" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="23" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F6" s="7">
@@ -1507,16 +1568,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="22" t="n">
         <v>46084</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="23" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F7" s="7">
@@ -1531,16 +1592,16 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="22" t="n">
         <v>46085</v>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C8" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="23" t="n">
         <v>0.6979166666666666</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F8" s="7">
@@ -1555,16 +1616,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="22" t="n">
         <v>46086</v>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C9" s="23" t="n">
         <v>0.3055555555555556</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="23" t="n">
         <v>0.6805555555555556</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F9" s="7">
@@ -1579,16 +1640,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="22" t="n">
         <v>46087</v>
       </c>
-      <c r="C10" s="19" t="n">
+      <c r="C10" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="23" t="n">
         <v>0.6736111111111112</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F10" s="7">
@@ -1598,58 +1659,58 @@
       <c r="G10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B11" s="20" t="n">
         <v>46088</v>
       </c>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B12" s="16" t="n">
+      <c r="B12" s="20" t="n">
         <v>46089</v>
       </c>
-      <c r="C12" s="15" t="n"/>
-      <c r="D12" s="15" t="n"/>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n"/>
-      <c r="G12" s="17" t="inlineStr">
+      <c r="C12" s="19" t="n"/>
+      <c r="D12" s="19" t="n"/>
+      <c r="E12" s="19" t="n"/>
+      <c r="F12" s="19" t="n"/>
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="n"/>
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="21" t="inlineStr">
+      <c r="A13" s="24" t="n"/>
+      <c r="B13" s="24" t="n"/>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="25" t="inlineStr">
         <is>
           <t>Summe KW 10</t>
         </is>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="26">
         <f>SUM(F6:F12)</f>
         <v/>
       </c>
-      <c r="G13" s="20" t="n"/>
+      <c r="G13" s="24" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1657,16 +1718,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="22" t="n">
         <v>46090</v>
       </c>
-      <c r="C14" s="19" t="n">
+      <c r="C14" s="23" t="n">
         <v>0.3125</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F14" s="7">
@@ -1681,16 +1742,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="22" t="n">
         <v>46091</v>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="23" t="n">
         <v>0.6701388888888888</v>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F15" s="7">
@@ -1705,16 +1766,16 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="22" t="n">
         <v>46092</v>
       </c>
-      <c r="C16" s="19" t="n">
+      <c r="C16" s="23" t="n">
         <v>0.3090277777777778</v>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="23" t="n">
         <v>0.6840277777777778</v>
       </c>
-      <c r="E16" s="19" t="n">
+      <c r="E16" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F16" s="7">
@@ -1729,16 +1790,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n">
+      <c r="B17" s="22" t="n">
         <v>46093</v>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="23" t="n">
         <v>0.6979166666666666</v>
       </c>
-      <c r="E17" s="19" t="n">
+      <c r="E17" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F17" s="7">
@@ -1753,16 +1814,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B18" s="18" t="n">
+      <c r="B18" s="22" t="n">
         <v>46094</v>
       </c>
-      <c r="C18" s="19" t="n">
+      <c r="C18" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D18" s="19" t="n">
+      <c r="D18" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="E18" s="19" t="n">
+      <c r="E18" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F18" s="7">
@@ -1772,58 +1833,58 @@
       <c r="G18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n">
+      <c r="B19" s="20" t="n">
         <v>46095</v>
       </c>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B20" s="16" t="n">
+      <c r="B20" s="20" t="n">
         <v>46096</v>
       </c>
-      <c r="C20" s="15" t="n"/>
-      <c r="D20" s="15" t="n"/>
-      <c r="E20" s="15" t="n"/>
-      <c r="F20" s="15" t="n"/>
-      <c r="G20" s="17" t="inlineStr">
+      <c r="C20" s="19" t="n"/>
+      <c r="D20" s="19" t="n"/>
+      <c r="E20" s="19" t="n"/>
+      <c r="F20" s="19" t="n"/>
+      <c r="G20" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="n"/>
-      <c r="B21" s="20" t="n"/>
-      <c r="C21" s="20" t="n"/>
-      <c r="D21" s="20" t="n"/>
-      <c r="E21" s="21" t="inlineStr">
+      <c r="A21" s="24" t="n"/>
+      <c r="B21" s="24" t="n"/>
+      <c r="C21" s="24" t="n"/>
+      <c r="D21" s="24" t="n"/>
+      <c r="E21" s="25" t="inlineStr">
         <is>
           <t>Summe KW 11</t>
         </is>
       </c>
-      <c r="F21" s="22">
+      <c r="F21" s="26">
         <f>SUM(F14:F20)</f>
         <v/>
       </c>
-      <c r="G21" s="20" t="n"/>
+      <c r="G21" s="24" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
@@ -1831,16 +1892,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B22" s="18" t="n">
+      <c r="B22" s="22" t="n">
         <v>46097</v>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C22" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D22" s="23" t="n">
         <v>0.6736111111111112</v>
       </c>
-      <c r="E22" s="19" t="n">
+      <c r="E22" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F22" s="7">
@@ -1855,16 +1916,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B23" s="18" t="n">
+      <c r="B23" s="22" t="n">
         <v>46098</v>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C23" s="23" t="n">
         <v>0.3055555555555556</v>
       </c>
-      <c r="D23" s="19" t="n">
+      <c r="D23" s="23" t="n">
         <v>0.6701388888888888</v>
       </c>
-      <c r="E23" s="19" t="n">
+      <c r="E23" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F23" s="7">
@@ -1879,13 +1940,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B24" s="18" t="n">
+      <c r="B24" s="22" t="n">
         <v>46099</v>
       </c>
-      <c r="C24" s="19" t="n">
+      <c r="C24" s="23" t="n">
         <v>0.5104166666666666</v>
       </c>
-      <c r="D24" s="19" t="n">
+      <c r="D24" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="E24" s="5" t="n"/>
@@ -1905,16 +1966,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B25" s="18" t="n">
+      <c r="B25" s="22" t="n">
         <v>46100</v>
       </c>
-      <c r="C25" s="19" t="n">
+      <c r="C25" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D25" s="19" t="n">
+      <c r="D25" s="23" t="n">
         <v>0.6597222222222222</v>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E25" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F25" s="7">
@@ -1924,77 +1985,77 @@
       <c r="G25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="B26" s="24" t="n">
+      <c r="B26" s="28" t="n">
         <v>46101</v>
       </c>
-      <c r="C26" s="23" t="n"/>
-      <c r="D26" s="23" t="n"/>
-      <c r="E26" s="23" t="n"/>
-      <c r="F26" s="23" t="n"/>
-      <c r="G26" s="25" t="inlineStr">
+      <c r="C26" s="27" t="n"/>
+      <c r="D26" s="27" t="n"/>
+      <c r="E26" s="27" t="n"/>
+      <c r="F26" s="27" t="n"/>
+      <c r="G26" s="29" t="inlineStr">
         <is>
           <t>Krank</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B27" s="16" t="n">
+      <c r="B27" s="20" t="n">
         <v>46102</v>
       </c>
-      <c r="C27" s="15" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="15" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="15" t="inlineStr">
+      <c r="A28" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B28" s="16" t="n">
+      <c r="B28" s="20" t="n">
         <v>46103</v>
       </c>
-      <c r="C28" s="15" t="n"/>
-      <c r="D28" s="15" t="n"/>
-      <c r="E28" s="15" t="n"/>
-      <c r="F28" s="15" t="n"/>
-      <c r="G28" s="17" t="inlineStr">
+      <c r="C28" s="19" t="n"/>
+      <c r="D28" s="19" t="n"/>
+      <c r="E28" s="19" t="n"/>
+      <c r="F28" s="19" t="n"/>
+      <c r="G28" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="20" t="n"/>
-      <c r="B29" s="20" t="n"/>
-      <c r="C29" s="20" t="n"/>
-      <c r="D29" s="20" t="n"/>
-      <c r="E29" s="21" t="inlineStr">
+      <c r="A29" s="24" t="n"/>
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="25" t="inlineStr">
         <is>
           <t>Summe KW 12</t>
         </is>
       </c>
-      <c r="F29" s="22">
+      <c r="F29" s="26">
         <f>SUM(F22:F28)</f>
         <v/>
       </c>
-      <c r="G29" s="20" t="n"/>
+      <c r="G29" s="24" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2002,16 +2063,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B30" s="18" t="n">
+      <c r="B30" s="22" t="n">
         <v>46104</v>
       </c>
-      <c r="C30" s="19" t="n">
+      <c r="C30" s="23" t="n">
         <v>0.3125</v>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D30" s="23" t="n">
         <v>0.6875</v>
       </c>
-      <c r="E30" s="19" t="n">
+      <c r="E30" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F30" s="7">
@@ -2026,16 +2087,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B31" s="18" t="n">
+      <c r="B31" s="22" t="n">
         <v>46105</v>
       </c>
-      <c r="C31" s="19" t="n">
+      <c r="C31" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D31" s="19" t="n">
+      <c r="D31" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="E31" s="19" t="n">
+      <c r="E31" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F31" s="7">
@@ -2050,13 +2111,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B32" s="18" t="n">
+      <c r="B32" s="22" t="n">
         <v>46106</v>
       </c>
-      <c r="C32" s="19" t="n">
+      <c r="C32" s="23" t="n">
         <v>0.5069444444444444</v>
       </c>
-      <c r="D32" s="19" t="n">
+      <c r="D32" s="23" t="n">
         <v>0.6736111111111112</v>
       </c>
       <c r="E32" s="5" t="n"/>
@@ -2076,16 +2137,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B33" s="18" t="n">
+      <c r="B33" s="22" t="n">
         <v>46107</v>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C33" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D33" s="19" t="n">
+      <c r="D33" s="23" t="n">
         <v>0.6979166666666666</v>
       </c>
-      <c r="E33" s="19" t="n">
+      <c r="E33" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F33" s="7">
@@ -2100,16 +2161,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B34" s="18" t="n">
+      <c r="B34" s="22" t="n">
         <v>46108</v>
       </c>
-      <c r="C34" s="19" t="n">
+      <c r="C34" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D34" s="19" t="n">
+      <c r="D34" s="23" t="n">
         <v>0.6701388888888888</v>
       </c>
-      <c r="E34" s="19" t="n">
+      <c r="E34" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F34" s="7">
@@ -2119,58 +2180,58 @@
       <c r="G34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B35" s="16" t="n">
+      <c r="B35" s="20" t="n">
         <v>46109</v>
       </c>
-      <c r="C35" s="15" t="n"/>
-      <c r="D35" s="15" t="n"/>
-      <c r="E35" s="15" t="n"/>
-      <c r="F35" s="15" t="n"/>
-      <c r="G35" s="17" t="inlineStr">
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="15" t="inlineStr">
+      <c r="A36" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B36" s="16" t="n">
+      <c r="B36" s="20" t="n">
         <v>46110</v>
       </c>
-      <c r="C36" s="15" t="n"/>
-      <c r="D36" s="15" t="n"/>
-      <c r="E36" s="15" t="n"/>
-      <c r="F36" s="15" t="n"/>
-      <c r="G36" s="17" t="inlineStr">
+      <c r="C36" s="19" t="n"/>
+      <c r="D36" s="19" t="n"/>
+      <c r="E36" s="19" t="n"/>
+      <c r="F36" s="19" t="n"/>
+      <c r="G36" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="20" t="n"/>
-      <c r="B37" s="20" t="n"/>
-      <c r="C37" s="20" t="n"/>
-      <c r="D37" s="20" t="n"/>
-      <c r="E37" s="21" t="inlineStr">
+      <c r="A37" s="24" t="n"/>
+      <c r="B37" s="24" t="n"/>
+      <c r="C37" s="24" t="n"/>
+      <c r="D37" s="24" t="n"/>
+      <c r="E37" s="25" t="inlineStr">
         <is>
           <t>Summe KW 13</t>
         </is>
       </c>
-      <c r="F37" s="22">
+      <c r="F37" s="26">
         <f>SUM(F30:F36)</f>
         <v/>
       </c>
-      <c r="G37" s="20" t="n"/>
+      <c r="G37" s="24" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -2178,16 +2239,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B38" s="18" t="n">
+      <c r="B38" s="22" t="n">
         <v>46111</v>
       </c>
-      <c r="C38" s="19" t="n">
+      <c r="C38" s="23" t="n">
         <v>0.3090277777777778</v>
       </c>
-      <c r="D38" s="19" t="n">
+      <c r="D38" s="23" t="n">
         <v>0.6736111111111112</v>
       </c>
-      <c r="E38" s="19" t="n">
+      <c r="E38" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F38" s="7">
@@ -2202,16 +2263,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B39" s="18" t="n">
+      <c r="B39" s="22" t="n">
         <v>46112</v>
       </c>
-      <c r="C39" s="19" t="n">
+      <c r="C39" s="23" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="D39" s="19" t="n">
+      <c r="D39" s="23" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E39" s="19" t="n">
+      <c r="E39" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F39" s="7">
@@ -2221,20 +2282,20 @@
       <c r="G39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="20" t="n"/>
-      <c r="B40" s="20" t="n"/>
-      <c r="C40" s="20" t="n"/>
-      <c r="D40" s="20" t="n"/>
-      <c r="E40" s="21" t="inlineStr">
+      <c r="A40" s="24" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="25" t="inlineStr">
         <is>
           <t>Summe KW 14</t>
         </is>
       </c>
-      <c r="F40" s="22">
+      <c r="F40" s="26">
         <f>SUM(F38:F39)</f>
         <v/>
       </c>
-      <c r="G40" s="26" t="inlineStr">
+      <c r="G40" s="30" t="inlineStr">
         <is>
           <t>anteilig – Woche reicht in den Nachbarmonat</t>
         </is>
@@ -2250,28 +2311,28 @@
         <f>F13+F21+F29+F37+F40</f>
         <v/>
       </c>
-      <c r="G41" s="27" t="inlineStr">
+      <c r="G41" s="31" t="inlineStr">
         <is>
           <t>Stunden netto im Monat</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="n"/>
-      <c r="B43" s="28" t="n"/>
-      <c r="C43" s="28" t="n"/>
-      <c r="E43" s="28" t="n"/>
-      <c r="F43" s="28" t="n"/>
-      <c r="G43" s="28" t="n"/>
-      <c r="H43" s="28" t="n"/>
+      <c r="A43" s="32" t="n"/>
+      <c r="B43" s="32" t="n"/>
+      <c r="C43" s="32" t="n"/>
+      <c r="E43" s="32" t="n"/>
+      <c r="F43" s="32" t="n"/>
+      <c r="G43" s="32" t="n"/>
+      <c r="H43" s="32" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="29" t="inlineStr">
+      <c r="A44" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift Praktikant</t>
         </is>
       </c>
-      <c r="E44" s="29" t="inlineStr">
+      <c r="E44" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift und Stempel des Betriebes</t>
         </is>
@@ -2374,13 +2435,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="22" t="n">
         <v>46113</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="23" t="n">
         <v>0.5138888888888888</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="23" t="n">
         <v>0.6805555555555556</v>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -2400,16 +2461,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="22" t="n">
         <v>46114</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="23" t="n">
         <v>0.3229166666666667</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="23" t="n">
         <v>0.6875</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F6" s="7">
@@ -2419,96 +2480,96 @@
       <c r="G6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="28" t="n">
         <v>46115</v>
       </c>
-      <c r="C7" s="23" t="n"/>
-      <c r="D7" s="23" t="n"/>
-      <c r="E7" s="23" t="n"/>
-      <c r="F7" s="23" t="n"/>
-      <c r="G7" s="25" t="inlineStr">
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="29" t="inlineStr">
         <is>
           <t>Karfreitag</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="20" t="n">
         <v>46116</v>
       </c>
-      <c r="C8" s="15" t="n"/>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="20" t="n">
         <v>46117</v>
       </c>
-      <c r="C9" s="15" t="n"/>
-      <c r="D9" s="15" t="n"/>
-      <c r="E9" s="15" t="n"/>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="20" t="n"/>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="21" t="inlineStr">
+      <c r="A10" s="24" t="n"/>
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="25" t="inlineStr">
         <is>
           <t>Summe KW 14</t>
         </is>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="26">
         <f>SUM(F5:F9)</f>
         <v/>
       </c>
-      <c r="G10" s="26" t="inlineStr">
+      <c r="G10" s="30" t="inlineStr">
         <is>
           <t>anteilig – Woche reicht in den Nachbarmonat</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="27" t="inlineStr">
         <is>
           <t>Mo</t>
         </is>
       </c>
-      <c r="B11" s="24" t="n">
+      <c r="B11" s="28" t="n">
         <v>46118</v>
       </c>
-      <c r="C11" s="23" t="n"/>
-      <c r="D11" s="23" t="n"/>
-      <c r="E11" s="23" t="n"/>
-      <c r="F11" s="23" t="n"/>
-      <c r="G11" s="25" t="inlineStr">
+      <c r="C11" s="27" t="n"/>
+      <c r="D11" s="27" t="n"/>
+      <c r="E11" s="27" t="n"/>
+      <c r="F11" s="27" t="n"/>
+      <c r="G11" s="29" t="inlineStr">
         <is>
           <t>Ostermontag</t>
         </is>
@@ -2520,16 +2581,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="22" t="n">
         <v>46119</v>
       </c>
-      <c r="C12" s="19" t="n">
+      <c r="C12" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D12" s="19" t="n">
+      <c r="D12" s="23" t="n">
         <v>0.6527777777777778</v>
       </c>
-      <c r="E12" s="19" t="n">
+      <c r="E12" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F12" s="7">
@@ -2544,13 +2605,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="22" t="n">
         <v>46120</v>
       </c>
-      <c r="C13" s="19" t="n">
+      <c r="C13" s="23" t="n">
         <v>0.5104166666666666</v>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="E13" s="5" t="n"/>
@@ -2570,16 +2631,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="22" t="n">
         <v>46121</v>
       </c>
-      <c r="C14" s="19" t="n">
+      <c r="C14" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F14" s="7">
@@ -2594,16 +2655,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="22" t="n">
         <v>46122</v>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="23" t="n">
         <v>0.3055555555555556</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="23" t="n">
         <v>0.6701388888888888</v>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F15" s="7">
@@ -2613,58 +2674,58 @@
       <c r="G15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B16" s="16" t="n">
+      <c r="B16" s="20" t="n">
         <v>46123</v>
       </c>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B17" s="16" t="n">
+      <c r="B17" s="20" t="n">
         <v>46124</v>
       </c>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="17" t="inlineStr">
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="n"/>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="A18" s="24" t="n"/>
+      <c r="B18" s="24" t="n"/>
+      <c r="C18" s="24" t="n"/>
+      <c r="D18" s="24" t="n"/>
+      <c r="E18" s="25" t="inlineStr">
         <is>
           <t>Summe KW 15</t>
         </is>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="26">
         <f>SUM(F11:F17)</f>
         <v/>
       </c>
-      <c r="G18" s="20" t="n"/>
+      <c r="G18" s="24" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -2672,16 +2733,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B19" s="18" t="n">
+      <c r="B19" s="22" t="n">
         <v>46125</v>
       </c>
-      <c r="C19" s="19" t="n">
+      <c r="C19" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D19" s="19" t="n">
+      <c r="D19" s="23" t="n">
         <v>0.6701388888888888</v>
       </c>
-      <c r="E19" s="19" t="n">
+      <c r="E19" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F19" s="7">
@@ -2696,16 +2757,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B20" s="18" t="n">
+      <c r="B20" s="22" t="n">
         <v>46126</v>
       </c>
-      <c r="C20" s="19" t="n">
+      <c r="C20" s="23" t="n">
         <v>0.3159722222222222</v>
       </c>
-      <c r="D20" s="19" t="n">
+      <c r="D20" s="23" t="n">
         <v>0.6701388888888888</v>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E20" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F20" s="7">
@@ -2720,13 +2781,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B21" s="18" t="n">
+      <c r="B21" s="22" t="n">
         <v>46127</v>
       </c>
-      <c r="C21" s="19" t="n">
+      <c r="C21" s="23" t="n">
         <v>0.5173611111111112</v>
       </c>
-      <c r="D21" s="19" t="n">
+      <c r="D21" s="23" t="n">
         <v>0.6840277777777778</v>
       </c>
       <c r="E21" s="5" t="n"/>
@@ -2746,16 +2807,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B22" s="18" t="n">
+      <c r="B22" s="22" t="n">
         <v>46128</v>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C22" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D22" s="23" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E22" s="19" t="n">
+      <c r="E22" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F22" s="7">
@@ -2770,16 +2831,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B23" s="18" t="n">
+      <c r="B23" s="22" t="n">
         <v>46129</v>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C23" s="23" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="D23" s="19" t="n">
+      <c r="D23" s="23" t="n">
         <v>0.65625</v>
       </c>
-      <c r="E23" s="19" t="n">
+      <c r="E23" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F23" s="7">
@@ -2789,58 +2850,58 @@
       <c r="G23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
+      <c r="B24" s="20" t="n">
         <v>46130</v>
       </c>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="17" t="inlineStr">
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B25" s="16" t="n">
+      <c r="B25" s="20" t="n">
         <v>46131</v>
       </c>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="17" t="inlineStr">
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="20" t="n"/>
-      <c r="C26" s="20" t="n"/>
-      <c r="D26" s="20" t="n"/>
-      <c r="E26" s="21" t="inlineStr">
+      <c r="A26" s="24" t="n"/>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="25" t="inlineStr">
         <is>
           <t>Summe KW 16</t>
         </is>
       </c>
-      <c r="F26" s="22">
+      <c r="F26" s="26">
         <f>SUM(F19:F25)</f>
         <v/>
       </c>
-      <c r="G26" s="20" t="n"/>
+      <c r="G26" s="24" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -2848,16 +2909,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B27" s="18" t="n">
+      <c r="B27" s="22" t="n">
         <v>46132</v>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="C27" s="23" t="n">
         <v>0.3125</v>
       </c>
-      <c r="D27" s="19" t="n">
+      <c r="D27" s="23" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E27" s="19" t="n">
+      <c r="E27" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F27" s="7">
@@ -2872,16 +2933,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B28" s="18" t="n">
+      <c r="B28" s="22" t="n">
         <v>46133</v>
       </c>
-      <c r="C28" s="19" t="n">
+      <c r="C28" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D28" s="19" t="n">
+      <c r="D28" s="23" t="n">
         <v>0.6875</v>
       </c>
-      <c r="E28" s="19" t="n">
+      <c r="E28" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F28" s="7">
@@ -2896,13 +2957,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B29" s="18" t="n">
+      <c r="B29" s="22" t="n">
         <v>46134</v>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C29" s="23" t="n">
         <v>0.5069444444444444</v>
       </c>
-      <c r="D29" s="19" t="n">
+      <c r="D29" s="23" t="n">
         <v>0.6736111111111112</v>
       </c>
       <c r="E29" s="5" t="n"/>
@@ -2922,16 +2983,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B30" s="18" t="n">
+      <c r="B30" s="22" t="n">
         <v>46135</v>
       </c>
-      <c r="C30" s="19" t="n">
+      <c r="C30" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D30" s="23" t="n">
         <v>0.6631944444444444</v>
       </c>
-      <c r="E30" s="19" t="n">
+      <c r="E30" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F30" s="7">
@@ -2946,16 +3007,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B31" s="18" t="n">
+      <c r="B31" s="22" t="n">
         <v>46136</v>
       </c>
-      <c r="C31" s="19" t="n">
+      <c r="C31" s="23" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="D31" s="19" t="n">
+      <c r="D31" s="23" t="n">
         <v>0.6458333333333334</v>
       </c>
-      <c r="E31" s="19" t="n">
+      <c r="E31" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F31" s="7">
@@ -2965,58 +3026,58 @@
       <c r="G31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="15" t="inlineStr">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B32" s="16" t="n">
+      <c r="B32" s="20" t="n">
         <v>46137</v>
       </c>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="15" t="n"/>
-      <c r="F32" s="15" t="n"/>
-      <c r="G32" s="17" t="inlineStr">
+      <c r="C32" s="19" t="n"/>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B33" s="16" t="n">
+      <c r="B33" s="20" t="n">
         <v>46138</v>
       </c>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="15" t="n"/>
-      <c r="F33" s="15" t="n"/>
-      <c r="G33" s="17" t="inlineStr">
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="n"/>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="19" t="n"/>
+      <c r="G33" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="20" t="n"/>
-      <c r="B34" s="20" t="n"/>
-      <c r="C34" s="20" t="n"/>
-      <c r="D34" s="20" t="n"/>
-      <c r="E34" s="21" t="inlineStr">
+      <c r="A34" s="24" t="n"/>
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="25" t="inlineStr">
         <is>
           <t>Summe KW 17</t>
         </is>
       </c>
-      <c r="F34" s="22">
+      <c r="F34" s="26">
         <f>SUM(F27:F33)</f>
         <v/>
       </c>
-      <c r="G34" s="20" t="n"/>
+      <c r="G34" s="24" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -3024,16 +3085,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B35" s="18" t="n">
+      <c r="B35" s="22" t="n">
         <v>46139</v>
       </c>
-      <c r="C35" s="19" t="n">
+      <c r="C35" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D35" s="19" t="n">
+      <c r="D35" s="23" t="n">
         <v>0.65625</v>
       </c>
-      <c r="E35" s="19" t="n">
+      <c r="E35" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F35" s="7">
@@ -3048,16 +3109,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B36" s="18" t="n">
+      <c r="B36" s="22" t="n">
         <v>46140</v>
       </c>
-      <c r="C36" s="19" t="n">
+      <c r="C36" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D36" s="19" t="n">
+      <c r="D36" s="23" t="n">
         <v>0.7083333333333334</v>
       </c>
-      <c r="E36" s="19" t="n">
+      <c r="E36" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F36" s="7">
@@ -3067,19 +3128,19 @@
       <c r="G36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="23" t="inlineStr">
+      <c r="A37" s="27" t="inlineStr">
         <is>
           <t>Mi</t>
         </is>
       </c>
-      <c r="B37" s="24" t="n">
+      <c r="B37" s="28" t="n">
         <v>46141</v>
       </c>
-      <c r="C37" s="23" t="n"/>
-      <c r="D37" s="23" t="n"/>
-      <c r="E37" s="23" t="n"/>
-      <c r="F37" s="23" t="n"/>
-      <c r="G37" s="25" t="inlineStr">
+      <c r="C37" s="27" t="n"/>
+      <c r="D37" s="27" t="n"/>
+      <c r="E37" s="27" t="n"/>
+      <c r="F37" s="27" t="n"/>
+      <c r="G37" s="29" t="inlineStr">
         <is>
           <t>Vorlesung PP und Praktikum RT an der OTH</t>
         </is>
@@ -3091,16 +3152,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B38" s="18" t="n">
+      <c r="B38" s="22" t="n">
         <v>46142</v>
       </c>
-      <c r="C38" s="19" t="n">
+      <c r="C38" s="23" t="n">
         <v>0.3055555555555556</v>
       </c>
-      <c r="D38" s="19" t="n">
+      <c r="D38" s="23" t="n">
         <v>0.6701388888888888</v>
       </c>
-      <c r="E38" s="19" t="n">
+      <c r="E38" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F38" s="7">
@@ -3110,20 +3171,20 @@
       <c r="G38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="n"/>
-      <c r="B39" s="20" t="n"/>
-      <c r="C39" s="20" t="n"/>
-      <c r="D39" s="20" t="n"/>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="A39" s="24" t="n"/>
+      <c r="B39" s="24" t="n"/>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="25" t="inlineStr">
         <is>
           <t>Summe KW 18</t>
         </is>
       </c>
-      <c r="F39" s="22">
+      <c r="F39" s="26">
         <f>SUM(F35:F38)</f>
         <v/>
       </c>
-      <c r="G39" s="20" t="n"/>
+      <c r="G39" s="24" t="n"/>
     </row>
     <row r="40">
       <c r="E40" s="9" t="inlineStr">
@@ -3135,28 +3196,28 @@
         <f>F10+F18+F26+F34+F39</f>
         <v/>
       </c>
-      <c r="G40" s="27" t="inlineStr">
+      <c r="G40" s="31" t="inlineStr">
         <is>
           <t>Stunden netto im Monat</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="28" t="n"/>
-      <c r="B42" s="28" t="n"/>
-      <c r="C42" s="28" t="n"/>
-      <c r="E42" s="28" t="n"/>
-      <c r="F42" s="28" t="n"/>
-      <c r="G42" s="28" t="n"/>
-      <c r="H42" s="28" t="n"/>
+      <c r="A42" s="32" t="n"/>
+      <c r="B42" s="32" t="n"/>
+      <c r="C42" s="32" t="n"/>
+      <c r="E42" s="32" t="n"/>
+      <c r="F42" s="32" t="n"/>
+      <c r="G42" s="32" t="n"/>
+      <c r="H42" s="32" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="29" t="inlineStr">
+      <c r="A43" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift Praktikant</t>
         </is>
       </c>
-      <c r="E43" s="29" t="inlineStr">
+      <c r="E43" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift und Stempel des Betriebes</t>
         </is>
@@ -3254,57 +3315,57 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="B5" s="24" t="n">
+      <c r="B5" s="28" t="n">
         <v>46143</v>
       </c>
-      <c r="C5" s="23" t="n"/>
-      <c r="D5" s="23" t="n"/>
-      <c r="E5" s="23" t="n"/>
-      <c r="F5" s="23" t="n"/>
-      <c r="G5" s="25" t="inlineStr">
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="27" t="n"/>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="29" t="inlineStr">
         <is>
           <t>Tag der Arbeit</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B6" s="16" t="n">
+      <c r="B6" s="20" t="n">
         <v>46144</v>
       </c>
-      <c r="C6" s="15" t="n"/>
-      <c r="D6" s="15" t="n"/>
-      <c r="E6" s="15" t="n"/>
-      <c r="F6" s="15" t="n"/>
-      <c r="G6" s="17" t="inlineStr">
+      <c r="C6" s="19" t="n"/>
+      <c r="D6" s="19" t="n"/>
+      <c r="E6" s="19" t="n"/>
+      <c r="F6" s="19" t="n"/>
+      <c r="G6" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="A7" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B7" s="16" t="n">
+      <c r="B7" s="20" t="n">
         <v>46145</v>
       </c>
-      <c r="C7" s="15" t="n"/>
-      <c r="D7" s="15" t="n"/>
-      <c r="E7" s="15" t="n"/>
-      <c r="F7" s="15" t="n"/>
-      <c r="G7" s="17" t="inlineStr">
+      <c r="C7" s="19" t="n"/>
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n"/>
+      <c r="F7" s="19" t="n"/>
+      <c r="G7" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
@@ -3316,16 +3377,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="22" t="n">
         <v>46146</v>
       </c>
-      <c r="C8" s="19" t="n">
+      <c r="C8" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="23" t="n">
         <v>0.6736111111111112</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F8" s="7">
@@ -3340,16 +3401,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="22" t="n">
         <v>46147</v>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C9" s="23" t="n">
         <v>0.3125</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="23" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F9" s="7">
@@ -3364,13 +3425,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="22" t="n">
         <v>46148</v>
       </c>
-      <c r="C10" s="19" t="n">
+      <c r="C10" s="23" t="n">
         <v>0.5104166666666666</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="E10" s="5" t="n"/>
@@ -3390,16 +3451,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="22" t="n">
         <v>46149</v>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C11" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="23" t="n">
         <v>0.6388888888888888</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F11" s="7">
@@ -3414,16 +3475,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="22" t="n">
         <v>46150</v>
       </c>
-      <c r="C12" s="19" t="n">
+      <c r="C12" s="23" t="n">
         <v>0.3090277777777778</v>
       </c>
-      <c r="D12" s="19" t="n">
+      <c r="D12" s="23" t="n">
         <v>0.6736111111111112</v>
       </c>
-      <c r="E12" s="19" t="n">
+      <c r="E12" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F12" s="7">
@@ -3433,58 +3494,58 @@
       <c r="G12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="15" t="inlineStr">
+      <c r="A13" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B13" s="16" t="n">
+      <c r="B13" s="20" t="n">
         <v>46151</v>
       </c>
-      <c r="C13" s="15" t="n"/>
-      <c r="D13" s="15" t="n"/>
-      <c r="E13" s="15" t="n"/>
-      <c r="F13" s="15" t="n"/>
-      <c r="G13" s="17" t="inlineStr">
+      <c r="C13" s="19" t="n"/>
+      <c r="D13" s="19" t="n"/>
+      <c r="E13" s="19" t="n"/>
+      <c r="F13" s="19" t="n"/>
+      <c r="G13" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="15" t="inlineStr">
+      <c r="A14" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B14" s="16" t="n">
+      <c r="B14" s="20" t="n">
         <v>46152</v>
       </c>
-      <c r="C14" s="15" t="n"/>
-      <c r="D14" s="15" t="n"/>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="15" t="n"/>
-      <c r="G14" s="17" t="inlineStr">
+      <c r="C14" s="19" t="n"/>
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n"/>
+      <c r="F14" s="19" t="n"/>
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="n"/>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="21" t="inlineStr">
+      <c r="A15" s="24" t="n"/>
+      <c r="B15" s="24" t="n"/>
+      <c r="C15" s="24" t="n"/>
+      <c r="D15" s="24" t="n"/>
+      <c r="E15" s="25" t="inlineStr">
         <is>
           <t>Summe KW 19</t>
         </is>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="26">
         <f>SUM(F8:F14)</f>
         <v/>
       </c>
-      <c r="G15" s="20" t="n"/>
+      <c r="G15" s="24" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -3492,16 +3553,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="22" t="n">
         <v>46153</v>
       </c>
-      <c r="C16" s="19" t="n">
+      <c r="C16" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="23" t="n">
         <v>0.6979166666666666</v>
       </c>
-      <c r="E16" s="19" t="n">
+      <c r="E16" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F16" s="7">
@@ -3516,16 +3577,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n">
+      <c r="B17" s="22" t="n">
         <v>46154</v>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="23" t="n">
         <v>0.6458333333333334</v>
       </c>
-      <c r="E17" s="19" t="n">
+      <c r="E17" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F17" s="7">
@@ -3540,13 +3601,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B18" s="18" t="n">
+      <c r="B18" s="22" t="n">
         <v>46155</v>
       </c>
-      <c r="C18" s="19" t="n">
+      <c r="C18" s="23" t="n">
         <v>0.5138888888888888</v>
       </c>
-      <c r="D18" s="19" t="n">
+      <c r="D18" s="23" t="n">
         <v>0.6805555555555556</v>
       </c>
       <c r="E18" s="5" t="n"/>
@@ -3561,19 +3622,19 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" s="27" t="inlineStr">
         <is>
           <t>Do</t>
         </is>
       </c>
-      <c r="B19" s="24" t="n">
+      <c r="B19" s="28" t="n">
         <v>46156</v>
       </c>
-      <c r="C19" s="23" t="n"/>
-      <c r="D19" s="23" t="n"/>
-      <c r="E19" s="23" t="n"/>
-      <c r="F19" s="23" t="n"/>
-      <c r="G19" s="25" t="inlineStr">
+      <c r="C19" s="27" t="n"/>
+      <c r="D19" s="27" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="27" t="n"/>
+      <c r="G19" s="29" t="inlineStr">
         <is>
           <t>Christi Himmelfahrt</t>
         </is>
@@ -3585,16 +3646,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B20" s="18" t="n">
+      <c r="B20" s="22" t="n">
         <v>46157</v>
       </c>
-      <c r="C20" s="19" t="n">
+      <c r="C20" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D20" s="19" t="n">
+      <c r="D20" s="23" t="n">
         <v>0.6423611111111112</v>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E20" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F20" s="7">
@@ -3604,58 +3665,58 @@
       <c r="G20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="15" t="inlineStr">
+      <c r="A21" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B21" s="16" t="n">
+      <c r="B21" s="20" t="n">
         <v>46158</v>
       </c>
-      <c r="C21" s="15" t="n"/>
-      <c r="D21" s="15" t="n"/>
-      <c r="E21" s="15" t="n"/>
-      <c r="F21" s="15" t="n"/>
-      <c r="G21" s="17" t="inlineStr">
+      <c r="C21" s="19" t="n"/>
+      <c r="D21" s="19" t="n"/>
+      <c r="E21" s="19" t="n"/>
+      <c r="F21" s="19" t="n"/>
+      <c r="G21" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="15" t="inlineStr">
+      <c r="A22" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B22" s="16" t="n">
+      <c r="B22" s="20" t="n">
         <v>46159</v>
       </c>
-      <c r="C22" s="15" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="15" t="n"/>
-      <c r="F22" s="15" t="n"/>
-      <c r="G22" s="17" t="inlineStr">
+      <c r="C22" s="19" t="n"/>
+      <c r="D22" s="19" t="n"/>
+      <c r="E22" s="19" t="n"/>
+      <c r="F22" s="19" t="n"/>
+      <c r="G22" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="n"/>
-      <c r="B23" s="20" t="n"/>
-      <c r="C23" s="20" t="n"/>
-      <c r="D23" s="20" t="n"/>
-      <c r="E23" s="21" t="inlineStr">
+      <c r="A23" s="24" t="n"/>
+      <c r="B23" s="24" t="n"/>
+      <c r="C23" s="24" t="n"/>
+      <c r="D23" s="24" t="n"/>
+      <c r="E23" s="25" t="inlineStr">
         <is>
           <t>Summe KW 20</t>
         </is>
       </c>
-      <c r="F23" s="22">
+      <c r="F23" s="26">
         <f>SUM(F16:F22)</f>
         <v/>
       </c>
-      <c r="G23" s="20" t="n"/>
+      <c r="G23" s="24" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
@@ -3663,16 +3724,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B24" s="18" t="n">
+      <c r="B24" s="22" t="n">
         <v>46160</v>
       </c>
-      <c r="C24" s="19" t="n">
+      <c r="C24" s="23" t="n">
         <v>0.3055555555555556</v>
       </c>
-      <c r="D24" s="19" t="n">
+      <c r="D24" s="23" t="n">
         <v>0.6805555555555556</v>
       </c>
-      <c r="E24" s="19" t="n">
+      <c r="E24" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F24" s="7">
@@ -3687,16 +3748,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B25" s="18" t="n">
+      <c r="B25" s="22" t="n">
         <v>46161</v>
       </c>
-      <c r="C25" s="19" t="n">
+      <c r="C25" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D25" s="19" t="n">
+      <c r="D25" s="23" t="n">
         <v>0.6388888888888888</v>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E25" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F25" s="7">
@@ -3706,19 +3767,19 @@
       <c r="G25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>Mi</t>
         </is>
       </c>
-      <c r="B26" s="24" t="n">
+      <c r="B26" s="28" t="n">
         <v>46162</v>
       </c>
-      <c r="C26" s="23" t="n"/>
-      <c r="D26" s="23" t="n"/>
-      <c r="E26" s="23" t="n"/>
-      <c r="F26" s="23" t="n"/>
-      <c r="G26" s="25" t="inlineStr">
+      <c r="C26" s="27" t="n"/>
+      <c r="D26" s="27" t="n"/>
+      <c r="E26" s="27" t="n"/>
+      <c r="F26" s="27" t="n"/>
+      <c r="G26" s="29" t="inlineStr">
         <is>
           <t>Vorlesung PP und Praktikum RT an der OTH</t>
         </is>
@@ -3730,16 +3791,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B27" s="18" t="n">
+      <c r="B27" s="22" t="n">
         <v>46163</v>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="C27" s="23" t="n">
         <v>0.3125</v>
       </c>
-      <c r="D27" s="19" t="n">
+      <c r="D27" s="23" t="n">
         <v>0.65625</v>
       </c>
-      <c r="E27" s="19" t="n">
+      <c r="E27" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F27" s="7">
@@ -3754,16 +3815,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B28" s="18" t="n">
+      <c r="B28" s="22" t="n">
         <v>46164</v>
       </c>
-      <c r="C28" s="19" t="n">
+      <c r="C28" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D28" s="19" t="n">
+      <c r="D28" s="23" t="n">
         <v>0.65625</v>
       </c>
-      <c r="E28" s="19" t="n">
+      <c r="E28" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F28" s="7">
@@ -3773,73 +3834,73 @@
       <c r="G28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="15" t="inlineStr">
+      <c r="A29" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B29" s="16" t="n">
+      <c r="B29" s="20" t="n">
         <v>46165</v>
       </c>
-      <c r="C29" s="15" t="n"/>
-      <c r="D29" s="15" t="n"/>
-      <c r="E29" s="15" t="n"/>
-      <c r="F29" s="15" t="n"/>
-      <c r="G29" s="17" t="inlineStr">
+      <c r="C29" s="19" t="n"/>
+      <c r="D29" s="19" t="n"/>
+      <c r="E29" s="19" t="n"/>
+      <c r="F29" s="19" t="n"/>
+      <c r="G29" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B30" s="16" t="n">
+      <c r="B30" s="20" t="n">
         <v>46166</v>
       </c>
-      <c r="C30" s="15" t="n"/>
-      <c r="D30" s="15" t="n"/>
-      <c r="E30" s="15" t="n"/>
-      <c r="F30" s="15" t="n"/>
-      <c r="G30" s="17" t="inlineStr">
+      <c r="C30" s="19" t="n"/>
+      <c r="D30" s="19" t="n"/>
+      <c r="E30" s="19" t="n"/>
+      <c r="F30" s="19" t="n"/>
+      <c r="G30" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="n"/>
-      <c r="B31" s="20" t="n"/>
-      <c r="C31" s="20" t="n"/>
-      <c r="D31" s="20" t="n"/>
-      <c r="E31" s="21" t="inlineStr">
+      <c r="A31" s="24" t="n"/>
+      <c r="B31" s="24" t="n"/>
+      <c r="C31" s="24" t="n"/>
+      <c r="D31" s="24" t="n"/>
+      <c r="E31" s="25" t="inlineStr">
         <is>
           <t>Summe KW 21</t>
         </is>
       </c>
-      <c r="F31" s="22">
+      <c r="F31" s="26">
         <f>SUM(F24:F30)</f>
         <v/>
       </c>
-      <c r="G31" s="20" t="n"/>
+      <c r="G31" s="24" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="inlineStr">
+      <c r="A32" s="27" t="inlineStr">
         <is>
           <t>Mo</t>
         </is>
       </c>
-      <c r="B32" s="24" t="n">
+      <c r="B32" s="28" t="n">
         <v>46167</v>
       </c>
-      <c r="C32" s="23" t="n"/>
-      <c r="D32" s="23" t="n"/>
-      <c r="E32" s="23" t="n"/>
-      <c r="F32" s="23" t="n"/>
-      <c r="G32" s="25" t="inlineStr">
+      <c r="C32" s="27" t="n"/>
+      <c r="D32" s="27" t="n"/>
+      <c r="E32" s="27" t="n"/>
+      <c r="F32" s="27" t="n"/>
+      <c r="G32" s="29" t="inlineStr">
         <is>
           <t>Pfingstmontag</t>
         </is>
@@ -3851,16 +3912,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B33" s="18" t="n">
+      <c r="B33" s="22" t="n">
         <v>46168</v>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C33" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D33" s="19" t="n">
+      <c r="D33" s="23" t="n">
         <v>0.6666666666666666</v>
       </c>
-      <c r="E33" s="19" t="n">
+      <c r="E33" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F33" s="7">
@@ -3870,19 +3931,19 @@
       <c r="G33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="23" t="inlineStr">
+      <c r="A34" s="27" t="inlineStr">
         <is>
           <t>Mi</t>
         </is>
       </c>
-      <c r="B34" s="24" t="n">
+      <c r="B34" s="28" t="n">
         <v>46169</v>
       </c>
-      <c r="C34" s="23" t="n"/>
-      <c r="D34" s="23" t="n"/>
-      <c r="E34" s="23" t="n"/>
-      <c r="F34" s="23" t="n"/>
-      <c r="G34" s="25" t="inlineStr">
+      <c r="C34" s="27" t="n"/>
+      <c r="D34" s="27" t="n"/>
+      <c r="E34" s="27" t="n"/>
+      <c r="F34" s="27" t="n"/>
+      <c r="G34" s="29" t="inlineStr">
         <is>
           <t>Vorlesung PP und Praktikum RT an der OTH</t>
         </is>
@@ -3894,16 +3955,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B35" s="18" t="n">
+      <c r="B35" s="22" t="n">
         <v>46170</v>
       </c>
-      <c r="C35" s="19" t="n">
+      <c r="C35" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D35" s="19" t="n">
+      <c r="D35" s="23" t="n">
         <v>0.6284722222222222</v>
       </c>
-      <c r="E35" s="19" t="n">
+      <c r="E35" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F35" s="7">
@@ -3918,16 +3979,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B36" s="18" t="n">
+      <c r="B36" s="22" t="n">
         <v>46171</v>
       </c>
-      <c r="C36" s="19" t="n">
+      <c r="C36" s="23" t="n">
         <v>0.3090277777777778</v>
       </c>
-      <c r="D36" s="19" t="n">
+      <c r="D36" s="23" t="n">
         <v>0.6631944444444444</v>
       </c>
-      <c r="E36" s="19" t="n">
+      <c r="E36" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F36" s="7">
@@ -3937,58 +3998,58 @@
       <c r="G36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="15" t="inlineStr">
+      <c r="A37" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B37" s="16" t="n">
+      <c r="B37" s="20" t="n">
         <v>46172</v>
       </c>
-      <c r="C37" s="15" t="n"/>
-      <c r="D37" s="15" t="n"/>
-      <c r="E37" s="15" t="n"/>
-      <c r="F37" s="15" t="n"/>
-      <c r="G37" s="17" t="inlineStr">
+      <c r="C37" s="19" t="n"/>
+      <c r="D37" s="19" t="n"/>
+      <c r="E37" s="19" t="n"/>
+      <c r="F37" s="19" t="n"/>
+      <c r="G37" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="15" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B38" s="16" t="n">
+      <c r="B38" s="20" t="n">
         <v>46173</v>
       </c>
-      <c r="C38" s="15" t="n"/>
-      <c r="D38" s="15" t="n"/>
-      <c r="E38" s="15" t="n"/>
-      <c r="F38" s="15" t="n"/>
-      <c r="G38" s="17" t="inlineStr">
+      <c r="C38" s="19" t="n"/>
+      <c r="D38" s="19" t="n"/>
+      <c r="E38" s="19" t="n"/>
+      <c r="F38" s="19" t="n"/>
+      <c r="G38" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="n"/>
-      <c r="B39" s="20" t="n"/>
-      <c r="C39" s="20" t="n"/>
-      <c r="D39" s="20" t="n"/>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="A39" s="24" t="n"/>
+      <c r="B39" s="24" t="n"/>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="25" t="inlineStr">
         <is>
           <t>Summe KW 22</t>
         </is>
       </c>
-      <c r="F39" s="22">
+      <c r="F39" s="26">
         <f>SUM(F32:F38)</f>
         <v/>
       </c>
-      <c r="G39" s="20" t="n"/>
+      <c r="G39" s="24" t="n"/>
     </row>
     <row r="40">
       <c r="E40" s="9" t="inlineStr">
@@ -4000,28 +4061,28 @@
         <f>F15+F23+F31+F39</f>
         <v/>
       </c>
-      <c r="G40" s="27" t="inlineStr">
+      <c r="G40" s="31" t="inlineStr">
         <is>
           <t>Stunden netto im Monat</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="28" t="n"/>
-      <c r="B42" s="28" t="n"/>
-      <c r="C42" s="28" t="n"/>
-      <c r="E42" s="28" t="n"/>
-      <c r="F42" s="28" t="n"/>
-      <c r="G42" s="28" t="n"/>
-      <c r="H42" s="28" t="n"/>
+      <c r="A42" s="32" t="n"/>
+      <c r="B42" s="32" t="n"/>
+      <c r="C42" s="32" t="n"/>
+      <c r="E42" s="32" t="n"/>
+      <c r="F42" s="32" t="n"/>
+      <c r="G42" s="32" t="n"/>
+      <c r="H42" s="32" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="29" t="inlineStr">
+      <c r="A43" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift Praktikant</t>
         </is>
       </c>
-      <c r="E43" s="29" t="inlineStr">
+      <c r="E43" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift und Stempel des Betriebes</t>
         </is>
@@ -4124,16 +4185,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="22" t="n">
         <v>46174</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="23" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="23" t="n">
         <v>0.6458333333333334</v>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F5" s="7">
@@ -4148,16 +4209,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="22" t="n">
         <v>46175</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="23" t="n">
         <v>0.3229166666666667</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="23" t="n">
         <v>0.6354166666666666</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F6" s="7">
@@ -4172,13 +4233,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="22" t="n">
         <v>46176</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="23" t="n">
         <v>0.5104166666666666</v>
       </c>
-      <c r="D7" s="19" t="n">
+      <c r="D7" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="E7" s="5" t="n"/>
@@ -4193,19 +4254,19 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Do</t>
         </is>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="28" t="n">
         <v>46177</v>
       </c>
-      <c r="C8" s="23" t="n"/>
-      <c r="D8" s="23" t="n"/>
-      <c r="E8" s="23" t="n"/>
-      <c r="F8" s="23" t="n"/>
-      <c r="G8" s="25" t="inlineStr">
+      <c r="C8" s="27" t="n"/>
+      <c r="D8" s="27" t="n"/>
+      <c r="E8" s="27" t="n"/>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="29" t="inlineStr">
         <is>
           <t>Fronleichnam</t>
         </is>
@@ -4217,16 +4278,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="22" t="n">
         <v>46178</v>
       </c>
-      <c r="C9" s="19" t="n">
+      <c r="C9" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D9" s="19" t="n">
+      <c r="D9" s="23" t="n">
         <v>0.6215277777777778</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F9" s="7">
@@ -4236,58 +4297,58 @@
       <c r="G9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="A10" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B10" s="16" t="n">
+      <c r="B10" s="20" t="n">
         <v>46179</v>
       </c>
-      <c r="C10" s="15" t="n"/>
-      <c r="D10" s="15" t="n"/>
-      <c r="E10" s="15" t="n"/>
-      <c r="F10" s="15" t="n"/>
-      <c r="G10" s="17" t="inlineStr">
+      <c r="C10" s="19" t="n"/>
+      <c r="D10" s="19" t="n"/>
+      <c r="E10" s="19" t="n"/>
+      <c r="F10" s="19" t="n"/>
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="15" t="inlineStr">
+      <c r="A11" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B11" s="16" t="n">
+      <c r="B11" s="20" t="n">
         <v>46180</v>
       </c>
-      <c r="C11" s="15" t="n"/>
-      <c r="D11" s="15" t="n"/>
-      <c r="E11" s="15" t="n"/>
-      <c r="F11" s="15" t="n"/>
-      <c r="G11" s="17" t="inlineStr">
+      <c r="C11" s="19" t="n"/>
+      <c r="D11" s="19" t="n"/>
+      <c r="E11" s="19" t="n"/>
+      <c r="F11" s="19" t="n"/>
+      <c r="G11" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="n"/>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="21" t="inlineStr">
+      <c r="A12" s="24" t="n"/>
+      <c r="B12" s="24" t="n"/>
+      <c r="C12" s="24" t="n"/>
+      <c r="D12" s="24" t="n"/>
+      <c r="E12" s="25" t="inlineStr">
         <is>
           <t>Summe KW 23</t>
         </is>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="26">
         <f>SUM(F5:F11)</f>
         <v/>
       </c>
-      <c r="G12" s="20" t="n"/>
+      <c r="G12" s="24" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -4295,16 +4356,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="22" t="n">
         <v>46181</v>
       </c>
-      <c r="C13" s="19" t="n">
+      <c r="C13" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="E13" s="19" t="n">
+      <c r="E13" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F13" s="7">
@@ -4319,16 +4380,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="22" t="n">
         <v>46182</v>
       </c>
-      <c r="C14" s="19" t="n">
+      <c r="C14" s="23" t="n">
         <v>0.3055555555555556</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="23" t="n">
         <v>0.6493055555555556</v>
       </c>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F14" s="7">
@@ -4343,13 +4404,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="22" t="n">
         <v>46183</v>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="23" t="n">
         <v>0.5069444444444444</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="23" t="n">
         <v>0.6736111111111112</v>
       </c>
       <c r="E15" s="5" t="n"/>
@@ -4369,16 +4430,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="22" t="n">
         <v>46184</v>
       </c>
-      <c r="C16" s="19" t="n">
+      <c r="C16" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="23" t="n">
         <v>0.6180555555555556</v>
       </c>
-      <c r="E16" s="19" t="n">
+      <c r="E16" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F16" s="7">
@@ -4393,16 +4454,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n">
+      <c r="B17" s="22" t="n">
         <v>46185</v>
       </c>
-      <c r="C17" s="19" t="n">
+      <c r="C17" s="23" t="n">
         <v>0.3159722222222222</v>
       </c>
-      <c r="D17" s="19" t="n">
+      <c r="D17" s="23" t="n">
         <v>0.6284722222222222</v>
       </c>
-      <c r="E17" s="19" t="n">
+      <c r="E17" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F17" s="7">
@@ -4412,58 +4473,58 @@
       <c r="G17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B18" s="16" t="n">
+      <c r="B18" s="20" t="n">
         <v>46186</v>
       </c>
-      <c r="C18" s="15" t="n"/>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="15" t="n"/>
-      <c r="F18" s="15" t="n"/>
-      <c r="G18" s="17" t="inlineStr">
+      <c r="C18" s="19" t="n"/>
+      <c r="D18" s="19" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n">
+      <c r="B19" s="20" t="n">
         <v>46187</v>
       </c>
-      <c r="C19" s="15" t="n"/>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="15" t="n"/>
-      <c r="F19" s="15" t="n"/>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="C19" s="19" t="n"/>
+      <c r="D19" s="19" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="n"/>
-      <c r="B20" s="20" t="n"/>
-      <c r="C20" s="20" t="n"/>
-      <c r="D20" s="20" t="n"/>
-      <c r="E20" s="21" t="inlineStr">
+      <c r="A20" s="24" t="n"/>
+      <c r="B20" s="24" t="n"/>
+      <c r="C20" s="24" t="n"/>
+      <c r="D20" s="24" t="n"/>
+      <c r="E20" s="25" t="inlineStr">
         <is>
           <t>Summe KW 24</t>
         </is>
       </c>
-      <c r="F20" s="22">
+      <c r="F20" s="26">
         <f>SUM(F13:F19)</f>
         <v/>
       </c>
-      <c r="G20" s="20" t="n"/>
+      <c r="G20" s="24" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -4471,16 +4532,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B21" s="18" t="n">
+      <c r="B21" s="22" t="n">
         <v>46188</v>
       </c>
-      <c r="C21" s="19" t="n">
+      <c r="C21" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D21" s="19" t="n">
+      <c r="D21" s="23" t="n">
         <v>0.65625</v>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E21" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F21" s="7">
@@ -4495,16 +4556,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B22" s="18" t="n">
+      <c r="B22" s="22" t="n">
         <v>46189</v>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C22" s="23" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D22" s="23" t="n">
         <v>0.625</v>
       </c>
-      <c r="E22" s="19" t="n">
+      <c r="E22" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F22" s="7">
@@ -4519,13 +4580,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B23" s="18" t="n">
+      <c r="B23" s="22" t="n">
         <v>46190</v>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C23" s="23" t="n">
         <v>0.5138888888888888</v>
       </c>
-      <c r="D23" s="19" t="n">
+      <c r="D23" s="23" t="n">
         <v>0.6805555555555556</v>
       </c>
       <c r="E23" s="5" t="n"/>
@@ -4545,16 +4606,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B24" s="18" t="n">
+      <c r="B24" s="22" t="n">
         <v>46191</v>
       </c>
-      <c r="C24" s="19" t="n">
+      <c r="C24" s="23" t="n">
         <v>0.3125</v>
       </c>
-      <c r="D24" s="19" t="n">
+      <c r="D24" s="23" t="n">
         <v>0.6458333333333334</v>
       </c>
-      <c r="E24" s="19" t="n">
+      <c r="E24" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F24" s="7">
@@ -4569,16 +4630,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B25" s="18" t="n">
+      <c r="B25" s="22" t="n">
         <v>46192</v>
       </c>
-      <c r="C25" s="19" t="n">
+      <c r="C25" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D25" s="19" t="n">
+      <c r="D25" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E25" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F25" s="7">
@@ -4588,58 +4649,58 @@
       <c r="G25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B26" s="16" t="n">
+      <c r="B26" s="20" t="n">
         <v>46193</v>
       </c>
-      <c r="C26" s="15" t="n"/>
-      <c r="D26" s="15" t="n"/>
-      <c r="E26" s="15" t="n"/>
-      <c r="F26" s="15" t="n"/>
-      <c r="G26" s="17" t="inlineStr">
+      <c r="C26" s="19" t="n"/>
+      <c r="D26" s="19" t="n"/>
+      <c r="E26" s="19" t="n"/>
+      <c r="F26" s="19" t="n"/>
+      <c r="G26" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="15" t="inlineStr">
+      <c r="A27" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B27" s="16" t="n">
+      <c r="B27" s="20" t="n">
         <v>46194</v>
       </c>
-      <c r="C27" s="15" t="n"/>
-      <c r="D27" s="15" t="n"/>
-      <c r="E27" s="15" t="n"/>
-      <c r="F27" s="15" t="n"/>
-      <c r="G27" s="17" t="inlineStr">
+      <c r="C27" s="19" t="n"/>
+      <c r="D27" s="19" t="n"/>
+      <c r="E27" s="19" t="n"/>
+      <c r="F27" s="19" t="n"/>
+      <c r="G27" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="n"/>
-      <c r="B28" s="20" t="n"/>
-      <c r="C28" s="20" t="n"/>
-      <c r="D28" s="20" t="n"/>
-      <c r="E28" s="21" t="inlineStr">
+      <c r="A28" s="24" t="n"/>
+      <c r="B28" s="24" t="n"/>
+      <c r="C28" s="24" t="n"/>
+      <c r="D28" s="24" t="n"/>
+      <c r="E28" s="25" t="inlineStr">
         <is>
           <t>Summe KW 25</t>
         </is>
       </c>
-      <c r="F28" s="22">
+      <c r="F28" s="26">
         <f>SUM(F21:F27)</f>
         <v/>
       </c>
-      <c r="G28" s="20" t="n"/>
+      <c r="G28" s="24" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -4647,16 +4708,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B29" s="18" t="n">
+      <c r="B29" s="22" t="n">
         <v>46195</v>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C29" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D29" s="19" t="n">
+      <c r="D29" s="23" t="n">
         <v>0.6215277777777778</v>
       </c>
-      <c r="E29" s="19" t="n">
+      <c r="E29" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F29" s="7">
@@ -4671,16 +4732,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B30" s="18" t="n">
+      <c r="B30" s="22" t="n">
         <v>46196</v>
       </c>
-      <c r="C30" s="19" t="n">
+      <c r="C30" s="23" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D30" s="23" t="n">
         <v>0.6145833333333334</v>
       </c>
-      <c r="E30" s="19" t="n">
+      <c r="E30" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F30" s="7">
@@ -4695,13 +4756,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B31" s="18" t="n">
+      <c r="B31" s="22" t="n">
         <v>46197</v>
       </c>
-      <c r="C31" s="19" t="n">
+      <c r="C31" s="23" t="n">
         <v>0.5104166666666666</v>
       </c>
-      <c r="D31" s="19" t="n">
+      <c r="D31" s="23" t="n">
         <v>0.6770833333333334</v>
       </c>
       <c r="E31" s="5" t="n"/>
@@ -4721,16 +4782,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B32" s="18" t="n">
+      <c r="B32" s="22" t="n">
         <v>46198</v>
       </c>
-      <c r="C32" s="19" t="n">
+      <c r="C32" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D32" s="19" t="n">
+      <c r="D32" s="23" t="n">
         <v>0.6458333333333334</v>
       </c>
-      <c r="E32" s="19" t="n">
+      <c r="E32" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F32" s="7">
@@ -4745,16 +4806,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B33" s="18" t="n">
+      <c r="B33" s="22" t="n">
         <v>46199</v>
       </c>
-      <c r="C33" s="19" t="n">
+      <c r="C33" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D33" s="19" t="n">
+      <c r="D33" s="23" t="n">
         <v>0.6875</v>
       </c>
-      <c r="E33" s="19" t="n">
+      <c r="E33" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F33" s="7">
@@ -4764,58 +4825,58 @@
       <c r="G33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="15" t="inlineStr">
+      <c r="A34" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B34" s="16" t="n">
+      <c r="B34" s="20" t="n">
         <v>46200</v>
       </c>
-      <c r="C34" s="15" t="n"/>
-      <c r="D34" s="15" t="n"/>
-      <c r="E34" s="15" t="n"/>
-      <c r="F34" s="15" t="n"/>
-      <c r="G34" s="17" t="inlineStr">
+      <c r="C34" s="19" t="n"/>
+      <c r="D34" s="19" t="n"/>
+      <c r="E34" s="19" t="n"/>
+      <c r="F34" s="19" t="n"/>
+      <c r="G34" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="15" t="inlineStr">
+      <c r="A35" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B35" s="16" t="n">
+      <c r="B35" s="20" t="n">
         <v>46201</v>
       </c>
-      <c r="C35" s="15" t="n"/>
-      <c r="D35" s="15" t="n"/>
-      <c r="E35" s="15" t="n"/>
-      <c r="F35" s="15" t="n"/>
-      <c r="G35" s="17" t="inlineStr">
+      <c r="C35" s="19" t="n"/>
+      <c r="D35" s="19" t="n"/>
+      <c r="E35" s="19" t="n"/>
+      <c r="F35" s="19" t="n"/>
+      <c r="G35" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="n"/>
-      <c r="B36" s="20" t="n"/>
-      <c r="C36" s="20" t="n"/>
-      <c r="D36" s="20" t="n"/>
-      <c r="E36" s="21" t="inlineStr">
+      <c r="A36" s="24" t="n"/>
+      <c r="B36" s="24" t="n"/>
+      <c r="C36" s="24" t="n"/>
+      <c r="D36" s="24" t="n"/>
+      <c r="E36" s="25" t="inlineStr">
         <is>
           <t>Summe KW 26</t>
         </is>
       </c>
-      <c r="F36" s="22">
+      <c r="F36" s="26">
         <f>SUM(F29:F35)</f>
         <v/>
       </c>
-      <c r="G36" s="20" t="n"/>
+      <c r="G36" s="24" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -4823,16 +4884,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B37" s="18" t="n">
+      <c r="B37" s="22" t="n">
         <v>46202</v>
       </c>
-      <c r="C37" s="19" t="n">
+      <c r="C37" s="23" t="n">
         <v>0.3055555555555556</v>
       </c>
-      <c r="D37" s="19" t="n">
+      <c r="D37" s="23" t="n">
         <v>0.6180555555555556</v>
       </c>
-      <c r="E37" s="19" t="n">
+      <c r="E37" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F37" s="7">
@@ -4847,16 +4908,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B38" s="18" t="n">
+      <c r="B38" s="22" t="n">
         <v>46203</v>
       </c>
-      <c r="C38" s="19" t="n">
+      <c r="C38" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D38" s="19" t="n">
+      <c r="D38" s="23" t="n">
         <v>0.6319444444444444</v>
       </c>
-      <c r="E38" s="19" t="n">
+      <c r="E38" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F38" s="7">
@@ -4866,20 +4927,20 @@
       <c r="G38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="n"/>
-      <c r="B39" s="20" t="n"/>
-      <c r="C39" s="20" t="n"/>
-      <c r="D39" s="20" t="n"/>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="A39" s="24" t="n"/>
+      <c r="B39" s="24" t="n"/>
+      <c r="C39" s="24" t="n"/>
+      <c r="D39" s="24" t="n"/>
+      <c r="E39" s="25" t="inlineStr">
         <is>
           <t>Summe KW 27</t>
         </is>
       </c>
-      <c r="F39" s="22">
+      <c r="F39" s="26">
         <f>SUM(F37:F38)</f>
         <v/>
       </c>
-      <c r="G39" s="26" t="inlineStr">
+      <c r="G39" s="30" t="inlineStr">
         <is>
           <t>anteilig – Woche reicht in den Nachbarmonat</t>
         </is>
@@ -4895,28 +4956,28 @@
         <f>F12+F20+F28+F36+F39</f>
         <v/>
       </c>
-      <c r="G40" s="27" t="inlineStr">
+      <c r="G40" s="31" t="inlineStr">
         <is>
           <t>Stunden netto im Monat</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="28" t="n"/>
-      <c r="B42" s="28" t="n"/>
-      <c r="C42" s="28" t="n"/>
-      <c r="E42" s="28" t="n"/>
-      <c r="F42" s="28" t="n"/>
-      <c r="G42" s="28" t="n"/>
-      <c r="H42" s="28" t="n"/>
+      <c r="A42" s="32" t="n"/>
+      <c r="B42" s="32" t="n"/>
+      <c r="C42" s="32" t="n"/>
+      <c r="E42" s="32" t="n"/>
+      <c r="F42" s="32" t="n"/>
+      <c r="G42" s="32" t="n"/>
+      <c r="H42" s="32" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="29" t="inlineStr">
+      <c r="A43" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift Praktikant</t>
         </is>
       </c>
-      <c r="E43" s="29" t="inlineStr">
+      <c r="E43" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift und Stempel des Betriebes</t>
         </is>
@@ -5019,13 +5080,13 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="22" t="n">
         <v>46204</v>
       </c>
-      <c r="C5" s="19" t="n">
+      <c r="C5" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D5" s="19" t="n">
+      <c r="D5" s="23" t="n">
         <v>0.5833333333333334</v>
       </c>
       <c r="E5" s="5" t="n"/>
@@ -5045,16 +5106,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="22" t="n">
         <v>46205</v>
       </c>
-      <c r="C6" s="19" t="n">
+      <c r="C6" s="23" t="n">
         <v>0.3125</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="23" t="n">
         <v>0.6458333333333334</v>
       </c>
-      <c r="E6" s="19" t="n">
+      <c r="E6" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F6" s="7">
@@ -5064,77 +5125,77 @@
       <c r="G6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>Fr</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="28" t="n">
         <v>46206</v>
       </c>
-      <c r="C7" s="23" t="n"/>
-      <c r="D7" s="23" t="n"/>
-      <c r="E7" s="23" t="n"/>
-      <c r="F7" s="23" t="n"/>
-      <c r="G7" s="25" t="inlineStr">
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="27" t="n"/>
+      <c r="E7" s="27" t="n"/>
+      <c r="F7" s="27" t="n"/>
+      <c r="G7" s="29" t="inlineStr">
         <is>
           <t>Krank</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B8" s="16" t="n">
+      <c r="B8" s="20" t="n">
         <v>46207</v>
       </c>
-      <c r="C8" s="15" t="n"/>
-      <c r="D8" s="15" t="n"/>
-      <c r="E8" s="15" t="n"/>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="17" t="inlineStr">
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n"/>
+      <c r="F8" s="19" t="n"/>
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B9" s="16" t="n">
+      <c r="B9" s="20" t="n">
         <v>46208</v>
       </c>
-      <c r="C9" s="15" t="n"/>
-      <c r="D9" s="15" t="n"/>
-      <c r="E9" s="15" t="n"/>
-      <c r="F9" s="15" t="n"/>
-      <c r="G9" s="17" t="inlineStr">
+      <c r="C9" s="19" t="n"/>
+      <c r="D9" s="19" t="n"/>
+      <c r="E9" s="19" t="n"/>
+      <c r="F9" s="19" t="n"/>
+      <c r="G9" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="20" t="n"/>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="21" t="inlineStr">
+      <c r="A10" s="24" t="n"/>
+      <c r="B10" s="24" t="n"/>
+      <c r="C10" s="24" t="n"/>
+      <c r="D10" s="24" t="n"/>
+      <c r="E10" s="25" t="inlineStr">
         <is>
           <t>Summe KW 27</t>
         </is>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="26">
         <f>SUM(F5:F9)</f>
         <v/>
       </c>
-      <c r="G10" s="26" t="inlineStr">
+      <c r="G10" s="30" t="inlineStr">
         <is>
           <t>anteilig – Woche reicht in den Nachbarmonat</t>
         </is>
@@ -5146,16 +5207,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="22" t="n">
         <v>46209</v>
       </c>
-      <c r="C11" s="19" t="n">
+      <c r="C11" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D11" s="19" t="n">
+      <c r="D11" s="23" t="n">
         <v>0.5868055555555556</v>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F11" s="7">
@@ -5170,16 +5231,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="22" t="n">
         <v>46210</v>
       </c>
-      <c r="C12" s="19" t="n">
+      <c r="C12" s="23" t="n">
         <v>0.3090277777777778</v>
       </c>
-      <c r="D12" s="19" t="n">
+      <c r="D12" s="23" t="n">
         <v>0.6111111111111112</v>
       </c>
-      <c r="E12" s="19" t="n">
+      <c r="E12" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F12" s="7">
@@ -5194,16 +5255,16 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="22" t="n">
         <v>46211</v>
       </c>
-      <c r="C13" s="19" t="n">
+      <c r="C13" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D13" s="19" t="n">
+      <c r="D13" s="23" t="n">
         <v>0.65625</v>
       </c>
-      <c r="E13" s="19" t="n">
+      <c r="E13" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F13" s="7">
@@ -5218,13 +5279,13 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="22" t="n">
         <v>46212</v>
       </c>
-      <c r="C14" s="19" t="n">
+      <c r="C14" s="23" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="D14" s="19" t="n">
+      <c r="D14" s="23" t="n">
         <v>0.625</v>
       </c>
       <c r="E14" s="5" t="n"/>
@@ -5244,16 +5305,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="22" t="n">
         <v>46213</v>
       </c>
-      <c r="C15" s="19" t="n">
+      <c r="C15" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D15" s="19" t="n">
+      <c r="D15" s="23" t="n">
         <v>0.625</v>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F15" s="7">
@@ -5263,58 +5324,58 @@
       <c r="G15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="15" t="inlineStr">
+      <c r="A16" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B16" s="16" t="n">
+      <c r="B16" s="20" t="n">
         <v>46214</v>
       </c>
-      <c r="C16" s="15" t="n"/>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n"/>
-      <c r="G16" s="17" t="inlineStr">
+      <c r="C16" s="19" t="n"/>
+      <c r="D16" s="19" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B17" s="16" t="n">
+      <c r="B17" s="20" t="n">
         <v>46215</v>
       </c>
-      <c r="C17" s="15" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="15" t="n"/>
-      <c r="F17" s="15" t="n"/>
-      <c r="G17" s="17" t="inlineStr">
+      <c r="C17" s="19" t="n"/>
+      <c r="D17" s="19" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="n"/>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="21" t="inlineStr">
+      <c r="A18" s="24" t="n"/>
+      <c r="B18" s="24" t="n"/>
+      <c r="C18" s="24" t="n"/>
+      <c r="D18" s="24" t="n"/>
+      <c r="E18" s="25" t="inlineStr">
         <is>
           <t>Summe KW 28</t>
         </is>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="26">
         <f>SUM(F11:F17)</f>
         <v/>
       </c>
-      <c r="G18" s="20" t="n"/>
+      <c r="G18" s="24" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -5322,16 +5383,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B19" s="18" t="n">
+      <c r="B19" s="22" t="n">
         <v>46216</v>
       </c>
-      <c r="C19" s="19" t="n">
+      <c r="C19" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D19" s="19" t="n">
+      <c r="D19" s="23" t="n">
         <v>0.6006944444444444</v>
       </c>
-      <c r="E19" s="19" t="n">
+      <c r="E19" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F19" s="7">
@@ -5346,16 +5407,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B20" s="18" t="n">
+      <c r="B20" s="22" t="n">
         <v>46217</v>
       </c>
-      <c r="C20" s="19" t="n">
+      <c r="C20" s="23" t="n">
         <v>0.3055555555555556</v>
       </c>
-      <c r="D20" s="19" t="n">
+      <c r="D20" s="23" t="n">
         <v>0.5972222222222222</v>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E20" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F20" s="7">
@@ -5370,16 +5431,16 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B21" s="18" t="n">
+      <c r="B21" s="22" t="n">
         <v>46218</v>
       </c>
-      <c r="C21" s="19" t="n">
+      <c r="C21" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D21" s="19" t="n">
+      <c r="D21" s="23" t="n">
         <v>0.6284722222222222</v>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E21" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F21" s="7">
@@ -5394,16 +5455,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B22" s="18" t="n">
+      <c r="B22" s="22" t="n">
         <v>46219</v>
       </c>
-      <c r="C22" s="19" t="n">
+      <c r="C22" s="23" t="n">
         <v>0.3125</v>
       </c>
-      <c r="D22" s="19" t="n">
+      <c r="D22" s="23" t="n">
         <v>0.625</v>
       </c>
-      <c r="E22" s="19" t="n">
+      <c r="E22" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F22" s="7">
@@ -5418,13 +5479,13 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B23" s="18" t="n">
+      <c r="B23" s="22" t="n">
         <v>46220</v>
       </c>
-      <c r="C23" s="19" t="n">
+      <c r="C23" s="23" t="n">
         <v>0.4618055555555556</v>
       </c>
-      <c r="D23" s="19" t="n">
+      <c r="D23" s="23" t="n">
         <v>0.6284722222222222</v>
       </c>
       <c r="E23" s="5" t="n"/>
@@ -5439,58 +5500,58 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B24" s="16" t="n">
+      <c r="B24" s="20" t="n">
         <v>46221</v>
       </c>
-      <c r="C24" s="15" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="15" t="n"/>
-      <c r="F24" s="15" t="n"/>
-      <c r="G24" s="17" t="inlineStr">
+      <c r="C24" s="19" t="n"/>
+      <c r="D24" s="19" t="n"/>
+      <c r="E24" s="19" t="n"/>
+      <c r="F24" s="19" t="n"/>
+      <c r="G24" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="15" t="inlineStr">
+      <c r="A25" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B25" s="16" t="n">
+      <c r="B25" s="20" t="n">
         <v>46222</v>
       </c>
-      <c r="C25" s="15" t="n"/>
-      <c r="D25" s="15" t="n"/>
-      <c r="E25" s="15" t="n"/>
-      <c r="F25" s="15" t="n"/>
-      <c r="G25" s="17" t="inlineStr">
+      <c r="C25" s="19" t="n"/>
+      <c r="D25" s="19" t="n"/>
+      <c r="E25" s="19" t="n"/>
+      <c r="F25" s="19" t="n"/>
+      <c r="G25" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="20" t="n"/>
-      <c r="C26" s="20" t="n"/>
-      <c r="D26" s="20" t="n"/>
-      <c r="E26" s="21" t="inlineStr">
+      <c r="A26" s="24" t="n"/>
+      <c r="B26" s="24" t="n"/>
+      <c r="C26" s="24" t="n"/>
+      <c r="D26" s="24" t="n"/>
+      <c r="E26" s="25" t="inlineStr">
         <is>
           <t>Summe KW 29</t>
         </is>
       </c>
-      <c r="F26" s="22">
+      <c r="F26" s="26">
         <f>SUM(F19:F25)</f>
         <v/>
       </c>
-      <c r="G26" s="20" t="n"/>
+      <c r="G26" s="24" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -5498,13 +5559,13 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B27" s="18" t="n">
+      <c r="B27" s="22" t="n">
         <v>46223</v>
       </c>
-      <c r="C27" s="19" t="n">
+      <c r="C27" s="23" t="n">
         <v>0.4583333333333333</v>
       </c>
-      <c r="D27" s="19" t="n">
+      <c r="D27" s="23" t="n">
         <v>0.625</v>
       </c>
       <c r="E27" s="5" t="n"/>
@@ -5524,16 +5585,16 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B28" s="18" t="n">
+      <c r="B28" s="22" t="n">
         <v>46224</v>
       </c>
-      <c r="C28" s="19" t="n">
+      <c r="C28" s="23" t="n">
         <v>0.3020833333333333</v>
       </c>
-      <c r="D28" s="19" t="n">
+      <c r="D28" s="23" t="n">
         <v>0.6145833333333334</v>
       </c>
-      <c r="E28" s="19" t="n">
+      <c r="E28" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F28" s="7">
@@ -5548,16 +5609,16 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B29" s="18" t="n">
+      <c r="B29" s="22" t="n">
         <v>46225</v>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C29" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D29" s="19" t="n">
+      <c r="D29" s="23" t="n">
         <v>0.65625</v>
       </c>
-      <c r="E29" s="19" t="n">
+      <c r="E29" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F29" s="7">
@@ -5572,16 +5633,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B30" s="18" t="n">
+      <c r="B30" s="22" t="n">
         <v>46226</v>
       </c>
-      <c r="C30" s="19" t="n">
+      <c r="C30" s="23" t="n">
         <v>0.2951388888888889</v>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D30" s="23" t="n">
         <v>0.5972222222222222</v>
       </c>
-      <c r="E30" s="19" t="n">
+      <c r="E30" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F30" s="7">
@@ -5596,16 +5657,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B31" s="18" t="n">
+      <c r="B31" s="22" t="n">
         <v>46227</v>
       </c>
-      <c r="C31" s="19" t="n">
+      <c r="C31" s="23" t="n">
         <v>0.3090277777777778</v>
       </c>
-      <c r="D31" s="19" t="n">
+      <c r="D31" s="23" t="n">
         <v>0.6111111111111112</v>
       </c>
-      <c r="E31" s="19" t="n">
+      <c r="E31" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F31" s="7">
@@ -5615,58 +5676,58 @@
       <c r="G31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="15" t="inlineStr">
+      <c r="A32" s="19" t="inlineStr">
         <is>
           <t>Sa</t>
         </is>
       </c>
-      <c r="B32" s="16" t="n">
+      <c r="B32" s="20" t="n">
         <v>46228</v>
       </c>
-      <c r="C32" s="15" t="n"/>
-      <c r="D32" s="15" t="n"/>
-      <c r="E32" s="15" t="n"/>
-      <c r="F32" s="15" t="n"/>
-      <c r="G32" s="17" t="inlineStr">
+      <c r="C32" s="19" t="n"/>
+      <c r="D32" s="19" t="n"/>
+      <c r="E32" s="19" t="n"/>
+      <c r="F32" s="19" t="n"/>
+      <c r="G32" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="15" t="inlineStr">
+      <c r="A33" s="19" t="inlineStr">
         <is>
           <t>So</t>
         </is>
       </c>
-      <c r="B33" s="16" t="n">
+      <c r="B33" s="20" t="n">
         <v>46229</v>
       </c>
-      <c r="C33" s="15" t="n"/>
-      <c r="D33" s="15" t="n"/>
-      <c r="E33" s="15" t="n"/>
-      <c r="F33" s="15" t="n"/>
-      <c r="G33" s="17" t="inlineStr">
+      <c r="C33" s="19" t="n"/>
+      <c r="D33" s="19" t="n"/>
+      <c r="E33" s="19" t="n"/>
+      <c r="F33" s="19" t="n"/>
+      <c r="G33" s="21" t="inlineStr">
         <is>
           <t>Wochenende</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="20" t="n"/>
-      <c r="B34" s="20" t="n"/>
-      <c r="C34" s="20" t="n"/>
-      <c r="D34" s="20" t="n"/>
-      <c r="E34" s="21" t="inlineStr">
+      <c r="A34" s="24" t="n"/>
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="25" t="inlineStr">
         <is>
           <t>Summe KW 30</t>
         </is>
       </c>
-      <c r="F34" s="22">
+      <c r="F34" s="26">
         <f>SUM(F27:F33)</f>
         <v/>
       </c>
-      <c r="G34" s="20" t="n"/>
+      <c r="G34" s="24" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -5674,16 +5735,16 @@
           <t>Mo</t>
         </is>
       </c>
-      <c r="B35" s="18" t="n">
+      <c r="B35" s="22" t="n">
         <v>46230</v>
       </c>
-      <c r="C35" s="19" t="n">
+      <c r="C35" s="23" t="n">
         <v>0.2916666666666667</v>
       </c>
-      <c r="D35" s="19" t="n">
+      <c r="D35" s="23" t="n">
         <v>0.6145833333333334</v>
       </c>
-      <c r="E35" s="19" t="n">
+      <c r="E35" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F35" s="7">
@@ -5698,13 +5759,13 @@
           <t>Di</t>
         </is>
       </c>
-      <c r="B36" s="18" t="n">
+      <c r="B36" s="22" t="n">
         <v>46231</v>
       </c>
-      <c r="C36" s="19" t="n">
+      <c r="C36" s="23" t="n">
         <v>0.4652777777777778</v>
       </c>
-      <c r="D36" s="19" t="n">
+      <c r="D36" s="23" t="n">
         <v>0.6319444444444444</v>
       </c>
       <c r="E36" s="5" t="n"/>
@@ -5724,16 +5785,16 @@
           <t>Mi</t>
         </is>
       </c>
-      <c r="B37" s="18" t="n">
+      <c r="B37" s="22" t="n">
         <v>46232</v>
       </c>
-      <c r="C37" s="19" t="n">
+      <c r="C37" s="23" t="n">
         <v>0.3229166666666667</v>
       </c>
-      <c r="D37" s="19" t="n">
+      <c r="D37" s="23" t="n">
         <v>0.65625</v>
       </c>
-      <c r="E37" s="19" t="n">
+      <c r="E37" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F37" s="7">
@@ -5748,16 +5809,16 @@
           <t>Do</t>
         </is>
       </c>
-      <c r="B38" s="18" t="n">
+      <c r="B38" s="22" t="n">
         <v>46233</v>
       </c>
-      <c r="C38" s="19" t="n">
+      <c r="C38" s="23" t="n">
         <v>0.2986111111111111</v>
       </c>
-      <c r="D38" s="19" t="n">
+      <c r="D38" s="23" t="n">
         <v>0.5902777777777778</v>
       </c>
-      <c r="E38" s="19" t="n">
+      <c r="E38" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F38" s="7">
@@ -5772,16 +5833,16 @@
           <t>Fr</t>
         </is>
       </c>
-      <c r="B39" s="18" t="n">
+      <c r="B39" s="22" t="n">
         <v>46234</v>
       </c>
-      <c r="C39" s="19" t="n">
+      <c r="C39" s="23" t="n">
         <v>0.3333333333333333</v>
       </c>
-      <c r="D39" s="19" t="n">
+      <c r="D39" s="23" t="n">
         <v>0.6458333333333334</v>
       </c>
-      <c r="E39" s="19" t="n">
+      <c r="E39" s="23" t="n">
         <v>0.02083333333333333</v>
       </c>
       <c r="F39" s="7">
@@ -5791,20 +5852,20 @@
       <c r="G39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="20" t="n"/>
-      <c r="B40" s="20" t="n"/>
-      <c r="C40" s="20" t="n"/>
-      <c r="D40" s="20" t="n"/>
-      <c r="E40" s="21" t="inlineStr">
+      <c r="A40" s="24" t="n"/>
+      <c r="B40" s="24" t="n"/>
+      <c r="C40" s="24" t="n"/>
+      <c r="D40" s="24" t="n"/>
+      <c r="E40" s="25" t="inlineStr">
         <is>
           <t>Summe KW 31</t>
         </is>
       </c>
-      <c r="F40" s="22">
+      <c r="F40" s="26">
         <f>SUM(F35:F39)</f>
         <v/>
       </c>
-      <c r="G40" s="20" t="n"/>
+      <c r="G40" s="24" t="n"/>
     </row>
     <row r="41">
       <c r="E41" s="9" t="inlineStr">
@@ -5816,28 +5877,28 @@
         <f>F10+F18+F26+F34+F40</f>
         <v/>
       </c>
-      <c r="G41" s="27" t="inlineStr">
+      <c r="G41" s="31" t="inlineStr">
         <is>
           <t>Stunden netto im Monat</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="n"/>
-      <c r="B43" s="28" t="n"/>
-      <c r="C43" s="28" t="n"/>
-      <c r="E43" s="28" t="n"/>
-      <c r="F43" s="28" t="n"/>
-      <c r="G43" s="28" t="n"/>
-      <c r="H43" s="28" t="n"/>
+      <c r="A43" s="32" t="n"/>
+      <c r="B43" s="32" t="n"/>
+      <c r="C43" s="32" t="n"/>
+      <c r="E43" s="32" t="n"/>
+      <c r="F43" s="32" t="n"/>
+      <c r="G43" s="32" t="n"/>
+      <c r="H43" s="32" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="29" t="inlineStr">
+      <c r="A44" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift Praktikant</t>
         </is>
       </c>
-      <c r="E44" s="29" t="inlineStr">
+      <c r="E44" s="33" t="inlineStr">
         <is>
           <t>Datum, Unterschrift und Stempel des Betriebes</t>
         </is>

</xml_diff>